<commit_message>
fix and update follow-up imagine
</commit_message>
<xml_diff>
--- a/output/results_0221_KB_review.xlsx
+++ b/output/results_0221_KB_review.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dulin/Dropbox/UTHealth/SAFElab/LLM/UTH_IPSS_Pediatric Stroke/Instructor/output/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dulin/Dropbox/UTHealth/SAFElab/LLM/UTH_IPSS_Pediatric Stroke/IPSS-GPT/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE84B3A8-1CE0-704B-A585-79D2CDE60E00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3606F145-785C-4440-A926-99D8294F4813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-36560" yWindow="-1240" windowWidth="38400" windowHeight="19900" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38400" yWindow="-1980" windowWidth="38400" windowHeight="19860" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PSOM_total (100% correct)" sheetId="1" r:id="rId1"/>
@@ -1468,7 +1468,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1539,7 +1539,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -4538,7 +4537,7 @@
       <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="27" t="s">
         <v>66</v>
       </c>
       <c r="D1" s="6" t="s">
@@ -5750,17 +5749,16 @@
       <c r="A6" s="3">
         <v>0</v>
       </c>
-      <c r="B6" s="28" t="s">
+      <c r="B6" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="28"/>
       <c r="D6" t="s">
         <v>140</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="I6" s="30" t="s">
+      <c r="I6" s="29" t="s">
         <v>386</v>
       </c>
       <c r="K6" t="s">
@@ -6410,7 +6408,7 @@
       <c r="H34" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="I34" s="29" t="s">
+      <c r="I34" s="28" t="s">
         <v>186</v>
       </c>
       <c r="K34" t="s">
@@ -6430,7 +6428,7 @@
       <c r="H35" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="I35" s="29" t="s">
+      <c r="I35" s="28" t="s">
         <v>156</v>
       </c>
       <c r="K35" t="s">
@@ -6511,7 +6509,7 @@
       <c r="H39" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="I39" s="29" t="s">
+      <c r="I39" s="28" t="s">
         <v>156</v>
       </c>
       <c r="K39" t="s">

</xml_diff>

<commit_message>
update neuro deficit type
</commit_message>
<xml_diff>
--- a/output/results_0221_KB_review.xlsx
+++ b/output/results_0221_KB_review.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dulin/Dropbox/UTHealth/SAFElab/LLM/UTH_IPSS_Pediatric Stroke/IPSS-GPT/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3606F145-785C-4440-A926-99D8294F4813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2DB5858-56C3-7E47-B534-68FB8531C517}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="-1980" windowWidth="38400" windowHeight="19860" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-34920" yWindow="-1400" windowWidth="18540" windowHeight="19860" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PSOM_total (100% correct)" sheetId="1" r:id="rId1"/>

</xml_diff>